<commit_message>
Creacion notebook procesamiento de datos de DANE y PDET
</commit_message>
<xml_diff>
--- a/semana_2/datos/raw/MunicipiosPDET.xlsx
+++ b/semana_2/datos/raw/MunicipiosPDET.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23801"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Juan Pablo\Proyecto-DBA\semana_2\datos\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7B3C975A-2454-4CFF-98FA-E66A81B079CF}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1C8C861-8B67-4F63-B1F9-8606960D9C82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MunicipiosPDET" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1031" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1031" uniqueCount="206">
   <si>
     <t>ALTO PATÍA Y NORTE DEL CAUCA</t>
   </si>
@@ -636,17 +636,20 @@
   </si>
   <si>
     <t>Municipio</t>
+  </si>
+  <si>
+    <t>CODDANEMuni</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="00000"/>
     <numFmt numFmtId="165" formatCode="00"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -777,6 +780,14 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1123,10 +1134,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1193,23 +1205,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:E171" totalsRowShown="0">
-  <autoFilter ref="A1:E171"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A1:E171" totalsRowShown="0">
+  <autoFilter ref="A1:E171" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" name="Subregión PDET"/>
-    <tableColumn id="2" name="Código DANE Departamento" dataDxfId="1"/>
-    <tableColumn id="3" name="Departamento"/>
-    <tableColumn id="4" name="Código DANE Municipio" dataDxfId="0"/>
-    <tableColumn id="5" name="Municipio"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Subregión PDET"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Código DANE Departamento" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Departamento"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="CODDANEMuni" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Municipio"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1247,7 +1259,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1353,7 +1365,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1495,25 +1507,25 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E171"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F171"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="45.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="45.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28" style="2" customWidth="1"/>
-    <col min="3" max="3" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.26953125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24" style="1" customWidth="1"/>
-    <col min="5" max="5" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>200</v>
       </c>
@@ -1524,13 +1536,13 @@
         <v>202</v>
       </c>
       <c r="D1" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E1" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1547,7 +1559,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1564,7 +1576,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -1581,7 +1593,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -1598,7 +1610,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -1614,8 +1626,9 @@
       <c r="E6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -1632,7 +1645,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -1649,7 +1662,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -1666,7 +1679,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -1683,7 +1696,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -1700,7 +1713,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -1717,7 +1730,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -1734,7 +1747,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -1751,7 +1764,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>0</v>
       </c>
@@ -1768,7 +1781,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>0</v>
       </c>
@@ -1785,7 +1798,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -1802,7 +1815,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -1819,7 +1832,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -1836,7 +1849,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>0</v>
       </c>
@@ -1853,7 +1866,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>0</v>
       </c>
@@ -1870,7 +1883,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>0</v>
       </c>
@@ -1887,7 +1900,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>0</v>
       </c>
@@ -1904,7 +1917,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -1921,7 +1934,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>0</v>
       </c>
@@ -1938,7 +1951,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>28</v>
       </c>
@@ -1955,7 +1968,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>28</v>
       </c>
@@ -1972,7 +1985,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>28</v>
       </c>
@@ -1989,7 +2002,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -2006,7 +2019,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>33</v>
       </c>
@@ -2023,7 +2036,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>33</v>
       </c>
@@ -2040,7 +2053,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>33</v>
       </c>
@@ -2057,7 +2070,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>33</v>
       </c>
@@ -2074,7 +2087,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>33</v>
       </c>
@@ -2091,7 +2104,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>33</v>
       </c>
@@ -2108,7 +2121,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>33</v>
       </c>
@@ -2125,7 +2138,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>33</v>
       </c>
@@ -2142,7 +2155,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>33</v>
       </c>
@@ -2159,7 +2172,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>33</v>
       </c>
@@ -2176,7 +2189,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>33</v>
       </c>
@@ -2193,7 +2206,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>33</v>
       </c>
@@ -2210,7 +2223,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>33</v>
       </c>
@@ -2227,7 +2240,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>48</v>
       </c>
@@ -2244,7 +2257,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>48</v>
       </c>
@@ -2261,7 +2274,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>48</v>
       </c>
@@ -2278,7 +2291,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>48</v>
       </c>
@@ -2295,7 +2308,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>48</v>
       </c>
@@ -2312,7 +2325,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>48</v>
       </c>
@@ -2329,7 +2342,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>48</v>
       </c>
@@ -2346,7 +2359,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>48</v>
       </c>
@@ -2363,7 +2376,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>58</v>
       </c>
@@ -2380,7 +2393,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>58</v>
       </c>
@@ -2397,7 +2410,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>58</v>
       </c>
@@ -2414,7 +2427,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>58</v>
       </c>
@@ -2431,7 +2444,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>58</v>
       </c>
@@ -2448,7 +2461,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>58</v>
       </c>
@@ -2465,7 +2478,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>58</v>
       </c>
@@ -2482,7 +2495,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>58</v>
       </c>
@@ -2499,7 +2512,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>58</v>
       </c>
@@ -2516,7 +2529,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>58</v>
       </c>
@@ -2533,7 +2546,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>58</v>
       </c>
@@ -2550,7 +2563,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>58</v>
       </c>
@@ -2567,7 +2580,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>58</v>
       </c>
@@ -2584,7 +2597,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>58</v>
       </c>
@@ -2601,7 +2614,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>73</v>
       </c>
@@ -2618,7 +2631,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>73</v>
       </c>
@@ -2635,7 +2648,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>73</v>
       </c>
@@ -2652,7 +2665,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>73</v>
       </c>
@@ -2669,7 +2682,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>73</v>
       </c>
@@ -2686,7 +2699,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>73</v>
       </c>
@@ -2703,7 +2716,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>73</v>
       </c>
@@ -2720,7 +2733,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>73</v>
       </c>
@@ -2737,7 +2750,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>73</v>
       </c>
@@ -2754,7 +2767,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>73</v>
       </c>
@@ -2771,7 +2784,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>73</v>
       </c>
@@ -2788,7 +2801,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>73</v>
       </c>
@@ -2805,7 +2818,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>73</v>
       </c>
@@ -2822,7 +2835,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>73</v>
       </c>
@@ -2839,7 +2852,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>73</v>
       </c>
@@ -2856,7 +2869,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>73</v>
       </c>
@@ -2873,7 +2886,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>73</v>
       </c>
@@ -2890,7 +2903,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>93</v>
       </c>
@@ -2907,7 +2920,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>93</v>
       </c>
@@ -2924,7 +2937,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>93</v>
       </c>
@@ -2941,7 +2954,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>93</v>
       </c>
@@ -2958,7 +2971,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>93</v>
       </c>
@@ -2975,7 +2988,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>93</v>
       </c>
@@ -2992,7 +3005,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>93</v>
       </c>
@@ -3009,7 +3022,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>93</v>
       </c>
@@ -3026,7 +3039,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>93</v>
       </c>
@@ -3043,7 +3056,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>93</v>
       </c>
@@ -3060,7 +3073,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>93</v>
       </c>
@@ -3077,7 +3090,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>93</v>
       </c>
@@ -3094,7 +3107,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>107</v>
       </c>
@@ -3111,7 +3124,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>107</v>
       </c>
@@ -3128,7 +3141,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>107</v>
       </c>
@@ -3145,7 +3158,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>107</v>
       </c>
@@ -3162,7 +3175,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>107</v>
       </c>
@@ -3179,7 +3192,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>107</v>
       </c>
@@ -3196,7 +3209,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>107</v>
       </c>
@@ -3213,7 +3226,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>107</v>
       </c>
@@ -3230,7 +3243,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>107</v>
       </c>
@@ -3247,7 +3260,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>107</v>
       </c>
@@ -3264,7 +3277,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>107</v>
       </c>
@@ -3281,7 +3294,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>107</v>
       </c>
@@ -3298,7 +3311,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>107</v>
       </c>
@@ -3315,7 +3328,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>107</v>
       </c>
@@ -3332,7 +3345,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>107</v>
       </c>
@@ -3349,7 +3362,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>125</v>
       </c>
@@ -3366,7 +3379,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>125</v>
       </c>
@@ -3383,7 +3396,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>125</v>
       </c>
@@ -3400,7 +3413,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>125</v>
       </c>
@@ -3417,7 +3430,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>130</v>
       </c>
@@ -3434,7 +3447,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>130</v>
       </c>
@@ -3451,7 +3464,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>130</v>
       </c>
@@ -3468,7 +3481,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>130</v>
       </c>
@@ -3485,7 +3498,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>130</v>
       </c>
@@ -3502,7 +3515,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>130</v>
       </c>
@@ -3519,7 +3532,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>130</v>
       </c>
@@ -3536,7 +3549,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>130</v>
       </c>
@@ -3553,7 +3566,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>130</v>
       </c>
@@ -3570,7 +3583,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>130</v>
       </c>
@@ -3587,7 +3600,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>130</v>
       </c>
@@ -3604,7 +3617,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>142</v>
       </c>
@@ -3621,7 +3634,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>142</v>
       </c>
@@ -3638,7 +3651,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>142</v>
       </c>
@@ -3655,7 +3668,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>142</v>
       </c>
@@ -3672,7 +3685,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>142</v>
       </c>
@@ -3689,7 +3702,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>142</v>
       </c>
@@ -3706,7 +3719,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>142</v>
       </c>
@@ -3723,7 +3736,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>142</v>
       </c>
@@ -3740,7 +3753,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>142</v>
       </c>
@@ -3757,7 +3770,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>152</v>
       </c>
@@ -3774,7 +3787,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>152</v>
       </c>
@@ -3791,7 +3804,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>152</v>
       </c>
@@ -3808,7 +3821,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>152</v>
       </c>
@@ -3825,7 +3838,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>152</v>
       </c>
@@ -3842,7 +3855,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>152</v>
       </c>
@@ -3859,7 +3872,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>152</v>
       </c>
@@ -3876,7 +3889,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>152</v>
       </c>
@@ -3893,7 +3906,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>152</v>
       </c>
@@ -3910,7 +3923,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>152</v>
       </c>
@@ -3927,7 +3940,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>152</v>
       </c>
@@ -3944,7 +3957,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>152</v>
       </c>
@@ -3961,7 +3974,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>152</v>
       </c>
@@ -3978,7 +3991,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>152</v>
       </c>
@@ -3995,7 +4008,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>152</v>
       </c>
@@ -4012,7 +4025,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>171</v>
       </c>
@@ -4029,7 +4042,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>171</v>
       </c>
@@ -4046,7 +4059,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>171</v>
       </c>
@@ -4063,7 +4076,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>171</v>
       </c>
@@ -4080,7 +4093,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>171</v>
       </c>
@@ -4097,7 +4110,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>171</v>
       </c>
@@ -4114,7 +4127,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>171</v>
       </c>
@@ -4131,7 +4144,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>178</v>
       </c>
@@ -4148,7 +4161,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>178</v>
       </c>
@@ -4165,7 +4178,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>178</v>
       </c>
@@ -4182,7 +4195,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>178</v>
       </c>
@@ -4199,7 +4212,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>178</v>
       </c>
@@ -4216,7 +4229,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>184</v>
       </c>
@@ -4233,7 +4246,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>184</v>
       </c>
@@ -4250,7 +4263,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>184</v>
       </c>
@@ -4267,7 +4280,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>184</v>
       </c>
@@ -4284,7 +4297,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>190</v>
       </c>
@@ -4301,7 +4314,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>190</v>
       </c>
@@ -4318,7 +4331,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>190</v>
       </c>
@@ -4335,7 +4348,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>190</v>
       </c>
@@ -4352,7 +4365,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>190</v>
       </c>
@@ -4369,7 +4382,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>190</v>
       </c>
@@ -4386,7 +4399,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>190</v>
       </c>
@@ -4403,7 +4416,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>190</v>
       </c>
@@ -4430,11 +4443,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F171"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>199</v>
       </c>
@@ -4454,7 +4467,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4474,7 +4487,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
@@ -4494,7 +4507,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1</v>
       </c>
@@ -4514,7 +4527,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1</v>
       </c>
@@ -4534,7 +4547,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1</v>
       </c>
@@ -4554,7 +4567,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1</v>
       </c>
@@ -4574,7 +4587,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1</v>
       </c>
@@ -4594,7 +4607,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1</v>
       </c>
@@ -4614,7 +4627,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>1</v>
       </c>
@@ -4634,7 +4647,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1</v>
       </c>
@@ -4654,7 +4667,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>1</v>
       </c>
@@ -4674,7 +4687,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1</v>
       </c>
@@ -4694,7 +4707,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>1</v>
       </c>
@@ -4714,7 +4727,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>1</v>
       </c>
@@ -4734,7 +4747,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>1</v>
       </c>
@@ -4754,7 +4767,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>1</v>
       </c>
@@ -4774,7 +4787,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>1</v>
       </c>
@@ -4794,7 +4807,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>1</v>
       </c>
@@ -4814,7 +4827,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>1</v>
       </c>
@@ -4834,7 +4847,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>1</v>
       </c>
@@ -4854,7 +4867,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>1</v>
       </c>
@@ -4874,7 +4887,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>1</v>
       </c>
@@ -4894,7 +4907,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>1</v>
       </c>
@@ -4914,7 +4927,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>1</v>
       </c>
@@ -4934,7 +4947,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>2</v>
       </c>
@@ -4954,7 +4967,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>2</v>
       </c>
@@ -4974,7 +4987,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>2</v>
       </c>
@@ -4994,7 +5007,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>2</v>
       </c>
@@ -5014,7 +5027,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>3</v>
       </c>
@@ -5034,7 +5047,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>3</v>
       </c>
@@ -5054,7 +5067,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>3</v>
       </c>
@@ -5074,7 +5087,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>3</v>
       </c>
@@ -5094,7 +5107,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>3</v>
       </c>
@@ -5114,7 +5127,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>3</v>
       </c>
@@ -5134,7 +5147,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>3</v>
       </c>
@@ -5154,7 +5167,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>3</v>
       </c>
@@ -5174,7 +5187,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>3</v>
       </c>
@@ -5194,7 +5207,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>3</v>
       </c>
@@ -5214,7 +5227,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>3</v>
       </c>
@@ -5234,7 +5247,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>3</v>
       </c>
@@ -5254,7 +5267,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>3</v>
       </c>
@@ -5274,7 +5287,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>4</v>
       </c>
@@ -5294,7 +5307,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>4</v>
       </c>
@@ -5314,7 +5327,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>4</v>
       </c>
@@ -5334,7 +5347,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>4</v>
       </c>
@@ -5354,7 +5367,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>4</v>
       </c>
@@ -5374,7 +5387,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>4</v>
       </c>
@@ -5394,7 +5407,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>4</v>
       </c>
@@ -5414,7 +5427,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>4</v>
       </c>
@@ -5434,7 +5447,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>5</v>
       </c>
@@ -5454,7 +5467,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>5</v>
       </c>
@@ -5474,7 +5487,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>5</v>
       </c>
@@ -5494,7 +5507,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>5</v>
       </c>
@@ -5514,7 +5527,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>5</v>
       </c>
@@ -5534,7 +5547,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>5</v>
       </c>
@@ -5554,7 +5567,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>5</v>
       </c>
@@ -5574,7 +5587,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>5</v>
       </c>
@@ -5594,7 +5607,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>5</v>
       </c>
@@ -5614,7 +5627,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>5</v>
       </c>
@@ -5634,7 +5647,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>5</v>
       </c>
@@ -5654,7 +5667,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>5</v>
       </c>
@@ -5674,7 +5687,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>5</v>
       </c>
@@ -5694,7 +5707,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>5</v>
       </c>
@@ -5714,7 +5727,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>6</v>
       </c>
@@ -5734,7 +5747,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>6</v>
       </c>
@@ -5754,7 +5767,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>6</v>
       </c>
@@ -5774,7 +5787,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>6</v>
       </c>
@@ -5794,7 +5807,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>6</v>
       </c>
@@ -5814,7 +5827,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>6</v>
       </c>
@@ -5834,7 +5847,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>6</v>
       </c>
@@ -5854,7 +5867,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>6</v>
       </c>
@@ -5874,7 +5887,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>6</v>
       </c>
@@ -5894,7 +5907,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>6</v>
       </c>
@@ -5914,7 +5927,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>6</v>
       </c>
@@ -5934,7 +5947,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>6</v>
       </c>
@@ -5954,7 +5967,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>6</v>
       </c>
@@ -5974,7 +5987,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>6</v>
       </c>
@@ -5994,7 +6007,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>6</v>
       </c>
@@ -6014,7 +6027,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>6</v>
       </c>
@@ -6034,7 +6047,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>6</v>
       </c>
@@ -6054,7 +6067,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>7</v>
       </c>
@@ -6074,7 +6087,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>7</v>
       </c>
@@ -6094,7 +6107,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>7</v>
       </c>
@@ -6114,7 +6127,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>7</v>
       </c>
@@ -6134,7 +6147,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>7</v>
       </c>
@@ -6154,7 +6167,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>7</v>
       </c>
@@ -6174,7 +6187,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>7</v>
       </c>
@@ -6194,7 +6207,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>7</v>
       </c>
@@ -6214,7 +6227,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>7</v>
       </c>
@@ -6234,7 +6247,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>7</v>
       </c>
@@ -6254,7 +6267,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>7</v>
       </c>
@@ -6274,7 +6287,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>7</v>
       </c>
@@ -6294,7 +6307,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>8</v>
       </c>
@@ -6314,7 +6327,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>8</v>
       </c>
@@ -6334,7 +6347,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>8</v>
       </c>
@@ -6354,7 +6367,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>8</v>
       </c>
@@ -6374,7 +6387,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>8</v>
       </c>
@@ -6394,7 +6407,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>8</v>
       </c>
@@ -6414,7 +6427,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>8</v>
       </c>
@@ -6434,7 +6447,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>8</v>
       </c>
@@ -6454,7 +6467,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>8</v>
       </c>
@@ -6474,7 +6487,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>8</v>
       </c>
@@ -6494,7 +6507,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>8</v>
       </c>
@@ -6514,7 +6527,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>8</v>
       </c>
@@ -6534,7 +6547,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>8</v>
       </c>
@@ -6554,7 +6567,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>8</v>
       </c>
@@ -6574,7 +6587,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>8</v>
       </c>
@@ -6594,7 +6607,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>9</v>
       </c>
@@ -6614,7 +6627,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>9</v>
       </c>
@@ -6634,7 +6647,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>9</v>
       </c>
@@ -6654,7 +6667,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>9</v>
       </c>
@@ -6674,7 +6687,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>10</v>
       </c>
@@ -6694,7 +6707,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>10</v>
       </c>
@@ -6714,7 +6727,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>10</v>
       </c>
@@ -6734,7 +6747,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>10</v>
       </c>
@@ -6754,7 +6767,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>10</v>
       </c>
@@ -6774,7 +6787,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>10</v>
       </c>
@@ -6794,7 +6807,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>10</v>
       </c>
@@ -6814,7 +6827,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>10</v>
       </c>
@@ -6834,7 +6847,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>10</v>
       </c>
@@ -6854,7 +6867,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>10</v>
       </c>
@@ -6874,7 +6887,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>10</v>
       </c>
@@ -6894,7 +6907,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>11</v>
       </c>
@@ -6914,7 +6927,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>11</v>
       </c>
@@ -6934,7 +6947,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>11</v>
       </c>
@@ -6954,7 +6967,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>11</v>
       </c>
@@ -6974,7 +6987,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>11</v>
       </c>
@@ -6994,7 +7007,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A129">
         <v>11</v>
       </c>
@@ -7014,7 +7027,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A130">
         <v>11</v>
       </c>
@@ -7034,7 +7047,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A131">
         <v>11</v>
       </c>
@@ -7054,7 +7067,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A132">
         <v>11</v>
       </c>
@@ -7074,7 +7087,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A133">
         <v>12</v>
       </c>
@@ -7094,7 +7107,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A134">
         <v>12</v>
       </c>
@@ -7114,7 +7127,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>12</v>
       </c>
@@ -7134,7 +7147,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A136">
         <v>12</v>
       </c>
@@ -7154,7 +7167,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A137">
         <v>12</v>
       </c>
@@ -7174,7 +7187,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A138">
         <v>12</v>
       </c>
@@ -7194,7 +7207,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A139">
         <v>12</v>
       </c>
@@ -7214,7 +7227,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A140">
         <v>12</v>
       </c>
@@ -7234,7 +7247,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A141">
         <v>12</v>
       </c>
@@ -7254,7 +7267,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A142">
         <v>12</v>
       </c>
@@ -7274,7 +7287,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A143">
         <v>12</v>
       </c>
@@ -7294,7 +7307,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A144">
         <v>12</v>
       </c>
@@ -7314,7 +7327,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A145">
         <v>12</v>
       </c>
@@ -7334,7 +7347,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A146">
         <v>12</v>
       </c>
@@ -7354,7 +7367,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A147">
         <v>12</v>
       </c>
@@ -7374,7 +7387,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A148">
         <v>13</v>
       </c>
@@ -7394,7 +7407,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A149">
         <v>13</v>
       </c>
@@ -7414,7 +7427,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A150">
         <v>13</v>
       </c>
@@ -7434,7 +7447,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A151">
         <v>13</v>
       </c>
@@ -7454,7 +7467,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A152">
         <v>13</v>
       </c>
@@ -7474,7 +7487,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A153">
         <v>13</v>
       </c>
@@ -7494,7 +7507,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A154">
         <v>13</v>
       </c>
@@ -7514,7 +7527,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A155">
         <v>14</v>
       </c>
@@ -7534,7 +7547,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A156">
         <v>14</v>
       </c>
@@ -7554,7 +7567,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A157">
         <v>14</v>
       </c>
@@ -7574,7 +7587,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A158">
         <v>14</v>
       </c>
@@ -7594,7 +7607,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A159">
         <v>14</v>
       </c>
@@ -7614,7 +7627,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A160">
         <v>15</v>
       </c>
@@ -7634,7 +7647,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A161">
         <v>15</v>
       </c>
@@ -7654,7 +7667,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A162">
         <v>15</v>
       </c>
@@ -7674,7 +7687,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A163">
         <v>15</v>
       </c>
@@ -7694,7 +7707,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A164">
         <v>16</v>
       </c>
@@ -7714,7 +7727,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A165">
         <v>16</v>
       </c>
@@ -7734,7 +7747,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A166">
         <v>16</v>
       </c>
@@ -7754,7 +7767,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A167">
         <v>16</v>
       </c>
@@ -7774,7 +7787,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A168">
         <v>16</v>
       </c>
@@ -7794,7 +7807,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A169">
         <v>16</v>
       </c>
@@ -7814,7 +7827,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A170">
         <v>16</v>
       </c>
@@ -7834,7 +7847,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A171">
         <v>16</v>
       </c>

</xml_diff>

<commit_message>
Script y geojson de municipios PDET procesados Corregido
</commit_message>
<xml_diff>
--- a/semana_2/datos/raw/MunicipiosPDET.xlsx
+++ b/semana_2/datos/raw/MunicipiosPDET.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Juan Pablo\Proyecto-DBA\semana_2\datos\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1C8C861-8B67-4F63-B1F9-8606960D9C82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C31C00D-EC40-41C0-9A6D-44FE38886573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1031" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1031" uniqueCount="208">
   <si>
     <t>ALTO PATÍA Y NORTE DEL CAUCA</t>
   </si>
@@ -638,15 +638,20 @@
     <t>Municipio</t>
   </si>
   <si>
-    <t>CODDANEMuni</t>
+    <t>CodMuni</t>
+  </si>
+  <si>
+    <t>CodDept</t>
+  </si>
+  <si>
+    <t>SubPDET</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="00000"/>
+  <numFmts count="1">
     <numFmt numFmtId="165" formatCode="00"/>
   </numFmts>
   <fonts count="19" x14ac:knownFonts="1">
@@ -1136,9 +1141,11 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1186,7 +1193,8 @@
   </cellStyles>
   <dxfs count="2">
     <dxf>
-      <numFmt numFmtId="164" formatCode="00000"/>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="165" formatCode="00"/>
@@ -1208,10 +1216,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A1:E171" totalsRowShown="0">
   <autoFilter ref="A1:E171" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Subregión PDET"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Código DANE Departamento" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SubPDET"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="CodDept" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Departamento"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="CODDANEMuni" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="CodMuni" dataDxfId="0"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Municipio"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1519,23 +1527,23 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="45.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28" style="2" customWidth="1"/>
+    <col min="2" max="2" width="28" style="1" customWidth="1"/>
     <col min="3" max="3" width="21.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24" style="1" customWidth="1"/>
+    <col min="4" max="4" width="24" style="3" customWidth="1"/>
     <col min="5" max="5" width="27.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="B1" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="C1" t="s">
         <v>202</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>205</v>
       </c>
       <c r="E1" t="s">
@@ -1546,13 +1554,13 @@
       <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>19</v>
       </c>
       <c r="C2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="3">
         <v>19050</v>
       </c>
       <c r="E2" t="s">
@@ -1563,13 +1571,13 @@
       <c r="A3" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>19</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="3">
         <v>19075</v>
       </c>
       <c r="E3" t="s">
@@ -1580,13 +1588,13 @@
       <c r="A4" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>19</v>
       </c>
       <c r="C4" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="3">
         <v>19110</v>
       </c>
       <c r="E4" t="s">
@@ -1597,13 +1605,13 @@
       <c r="A5" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>19</v>
       </c>
       <c r="C5" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="3">
         <v>19130</v>
       </c>
       <c r="E5" t="s">
@@ -1614,31 +1622,31 @@
       <c r="A6" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="1">
         <v>19</v>
       </c>
       <c r="C6" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="3">
         <v>19137</v>
       </c>
       <c r="E6" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="3"/>
+      <c r="F6" s="2"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="1">
         <v>19</v>
       </c>
       <c r="C7" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="3">
         <v>19142</v>
       </c>
       <c r="E7" t="s">
@@ -1649,13 +1657,13 @@
       <c r="A8" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="1">
         <v>19</v>
       </c>
       <c r="C8" t="s">
         <v>1</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="3">
         <v>19212</v>
       </c>
       <c r="E8" t="s">
@@ -1666,13 +1674,13 @@
       <c r="A9" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="1">
         <v>19</v>
       </c>
       <c r="C9" t="s">
         <v>1</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="3">
         <v>19256</v>
       </c>
       <c r="E9" t="s">
@@ -1683,13 +1691,13 @@
       <c r="A10" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="1">
         <v>19</v>
       </c>
       <c r="C10" t="s">
         <v>1</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="3">
         <v>19364</v>
       </c>
       <c r="E10" t="s">
@@ -1700,13 +1708,13 @@
       <c r="A11" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="1">
         <v>19</v>
       </c>
       <c r="C11" t="s">
         <v>1</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" s="3">
         <v>19450</v>
       </c>
       <c r="E11" t="s">
@@ -1717,13 +1725,13 @@
       <c r="A12" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="1">
         <v>19</v>
       </c>
       <c r="C12" t="s">
         <v>1</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="3">
         <v>19455</v>
       </c>
       <c r="E12" t="s">
@@ -1734,13 +1742,13 @@
       <c r="A13" t="s">
         <v>0</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="1">
         <v>19</v>
       </c>
       <c r="C13" t="s">
         <v>1</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="3">
         <v>19473</v>
       </c>
       <c r="E13" t="s">
@@ -1751,13 +1759,13 @@
       <c r="A14" t="s">
         <v>0</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14" s="1">
         <v>19</v>
       </c>
       <c r="C14" t="s">
         <v>1</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="3">
         <v>19532</v>
       </c>
       <c r="E14" t="s">
@@ -1768,13 +1776,13 @@
       <c r="A15" t="s">
         <v>0</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" s="1">
         <v>19</v>
       </c>
       <c r="C15" t="s">
         <v>1</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="3">
         <v>19548</v>
       </c>
       <c r="E15" t="s">
@@ -1785,13 +1793,13 @@
       <c r="A16" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="1">
         <v>19</v>
       </c>
       <c r="C16" t="s">
         <v>1</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="3">
         <v>19698</v>
       </c>
       <c r="E16" t="s">
@@ -1802,13 +1810,13 @@
       <c r="A17" t="s">
         <v>0</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="1">
         <v>19</v>
       </c>
       <c r="C17" t="s">
         <v>1</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="3">
         <v>19780</v>
       </c>
       <c r="E17" t="s">
@@ -1819,13 +1827,13 @@
       <c r="A18" t="s">
         <v>0</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="1">
         <v>19</v>
       </c>
       <c r="C18" t="s">
         <v>1</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="3">
         <v>19821</v>
       </c>
       <c r="E18" t="s">
@@ -1836,13 +1844,13 @@
       <c r="A19" t="s">
         <v>0</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="1">
         <v>52</v>
       </c>
       <c r="C19" t="s">
         <v>19</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="3">
         <v>52233</v>
       </c>
       <c r="E19" t="s">
@@ -1853,13 +1861,13 @@
       <c r="A20" t="s">
         <v>0</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20" s="1">
         <v>52</v>
       </c>
       <c r="C20" t="s">
         <v>19</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="3">
         <v>52256</v>
       </c>
       <c r="E20" t="s">
@@ -1870,13 +1878,13 @@
       <c r="A21" t="s">
         <v>0</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="1">
         <v>52</v>
       </c>
       <c r="C21" t="s">
         <v>19</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="3">
         <v>52405</v>
       </c>
       <c r="E21" t="s">
@@ -1887,13 +1895,13 @@
       <c r="A22" t="s">
         <v>0</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="1">
         <v>52</v>
       </c>
       <c r="C22" t="s">
         <v>19</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="3">
         <v>52418</v>
       </c>
       <c r="E22" t="s">
@@ -1904,13 +1912,13 @@
       <c r="A23" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="1">
         <v>52</v>
       </c>
       <c r="C23" t="s">
         <v>19</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="3">
         <v>52540</v>
       </c>
       <c r="E23" t="s">
@@ -1921,13 +1929,13 @@
       <c r="A24" t="s">
         <v>0</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24" s="1">
         <v>76</v>
       </c>
       <c r="C24" t="s">
         <v>25</v>
       </c>
-      <c r="D24" s="1">
+      <c r="D24" s="3">
         <v>76275</v>
       </c>
       <c r="E24" t="s">
@@ -1938,13 +1946,13 @@
       <c r="A25" t="s">
         <v>0</v>
       </c>
-      <c r="B25" s="2">
+      <c r="B25" s="1">
         <v>76</v>
       </c>
       <c r="C25" t="s">
         <v>25</v>
       </c>
-      <c r="D25" s="1">
+      <c r="D25" s="3">
         <v>76563</v>
       </c>
       <c r="E25" t="s">
@@ -1955,13 +1963,13 @@
       <c r="A26" t="s">
         <v>28</v>
       </c>
-      <c r="B26" s="2">
+      <c r="B26" s="1">
         <v>81</v>
       </c>
       <c r="C26" t="s">
         <v>28</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="3">
         <v>81065</v>
       </c>
       <c r="E26" t="s">
@@ -1972,13 +1980,13 @@
       <c r="A27" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="2">
+      <c r="B27" s="1">
         <v>81</v>
       </c>
       <c r="C27" t="s">
         <v>28</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="3">
         <v>81300</v>
       </c>
       <c r="E27" t="s">
@@ -1989,13 +1997,13 @@
       <c r="A28" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="2">
+      <c r="B28" s="1">
         <v>81</v>
       </c>
       <c r="C28" t="s">
         <v>28</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D28" s="3">
         <v>81736</v>
       </c>
       <c r="E28" t="s">
@@ -2006,13 +2014,13 @@
       <c r="A29" t="s">
         <v>28</v>
       </c>
-      <c r="B29" s="2">
+      <c r="B29" s="1">
         <v>81</v>
       </c>
       <c r="C29" t="s">
         <v>28</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="3">
         <v>81794</v>
       </c>
       <c r="E29" t="s">
@@ -2023,13 +2031,13 @@
       <c r="A30" t="s">
         <v>33</v>
       </c>
-      <c r="B30" s="2">
+      <c r="B30" s="1">
         <v>5</v>
       </c>
       <c r="C30" t="s">
         <v>34</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="3">
         <v>5031</v>
       </c>
       <c r="E30" t="s">
@@ -2040,13 +2048,13 @@
       <c r="A31" t="s">
         <v>33</v>
       </c>
-      <c r="B31" s="2">
+      <c r="B31" s="1">
         <v>5</v>
       </c>
       <c r="C31" t="s">
         <v>34</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="3">
         <v>5040</v>
       </c>
       <c r="E31" t="s">
@@ -2057,13 +2065,13 @@
       <c r="A32" t="s">
         <v>33</v>
       </c>
-      <c r="B32" s="2">
+      <c r="B32" s="1">
         <v>5</v>
       </c>
       <c r="C32" t="s">
         <v>34</v>
       </c>
-      <c r="D32" s="1">
+      <c r="D32" s="3">
         <v>5107</v>
       </c>
       <c r="E32" t="s">
@@ -2074,13 +2082,13 @@
       <c r="A33" t="s">
         <v>33</v>
       </c>
-      <c r="B33" s="2">
+      <c r="B33" s="1">
         <v>5</v>
       </c>
       <c r="C33" t="s">
         <v>34</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="3">
         <v>5120</v>
       </c>
       <c r="E33" t="s">
@@ -2091,13 +2099,13 @@
       <c r="A34" t="s">
         <v>33</v>
       </c>
-      <c r="B34" s="2">
+      <c r="B34" s="1">
         <v>5</v>
       </c>
       <c r="C34" t="s">
         <v>34</v>
       </c>
-      <c r="D34" s="1">
+      <c r="D34" s="3">
         <v>5154</v>
       </c>
       <c r="E34" t="s">
@@ -2108,13 +2116,13 @@
       <c r="A35" t="s">
         <v>33</v>
       </c>
-      <c r="B35" s="2">
+      <c r="B35" s="1">
         <v>5</v>
       </c>
       <c r="C35" t="s">
         <v>34</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="3">
         <v>5250</v>
       </c>
       <c r="E35" t="s">
@@ -2125,13 +2133,13 @@
       <c r="A36" t="s">
         <v>33</v>
       </c>
-      <c r="B36" s="2">
+      <c r="B36" s="1">
         <v>5</v>
       </c>
       <c r="C36" t="s">
         <v>34</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="3">
         <v>5361</v>
       </c>
       <c r="E36" t="s">
@@ -2142,13 +2150,13 @@
       <c r="A37" t="s">
         <v>33</v>
       </c>
-      <c r="B37" s="2">
+      <c r="B37" s="1">
         <v>5</v>
       </c>
       <c r="C37" t="s">
         <v>34</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="3">
         <v>5495</v>
       </c>
       <c r="E37" t="s">
@@ -2159,13 +2167,13 @@
       <c r="A38" t="s">
         <v>33</v>
       </c>
-      <c r="B38" s="2">
+      <c r="B38" s="1">
         <v>5</v>
       </c>
       <c r="C38" t="s">
         <v>34</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="3">
         <v>5604</v>
       </c>
       <c r="E38" t="s">
@@ -2176,13 +2184,13 @@
       <c r="A39" t="s">
         <v>33</v>
       </c>
-      <c r="B39" s="2">
+      <c r="B39" s="1">
         <v>5</v>
       </c>
       <c r="C39" t="s">
         <v>34</v>
       </c>
-      <c r="D39" s="1">
+      <c r="D39" s="3">
         <v>5736</v>
       </c>
       <c r="E39" t="s">
@@ -2193,13 +2201,13 @@
       <c r="A40" t="s">
         <v>33</v>
       </c>
-      <c r="B40" s="2">
+      <c r="B40" s="1">
         <v>5</v>
       </c>
       <c r="C40" t="s">
         <v>34</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="3">
         <v>5790</v>
       </c>
       <c r="E40" t="s">
@@ -2210,13 +2218,13 @@
       <c r="A41" t="s">
         <v>33</v>
       </c>
-      <c r="B41" s="2">
+      <c r="B41" s="1">
         <v>5</v>
       </c>
       <c r="C41" t="s">
         <v>34</v>
       </c>
-      <c r="D41" s="1">
+      <c r="D41" s="3">
         <v>5854</v>
       </c>
       <c r="E41" t="s">
@@ -2227,13 +2235,13 @@
       <c r="A42" t="s">
         <v>33</v>
       </c>
-      <c r="B42" s="2">
+      <c r="B42" s="1">
         <v>5</v>
       </c>
       <c r="C42" t="s">
         <v>34</v>
       </c>
-      <c r="D42" s="1">
+      <c r="D42" s="3">
         <v>5895</v>
       </c>
       <c r="E42" t="s">
@@ -2244,13 +2252,13 @@
       <c r="A43" t="s">
         <v>48</v>
       </c>
-      <c r="B43" s="2">
+      <c r="B43" s="1">
         <v>54</v>
       </c>
       <c r="C43" t="s">
         <v>49</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="3">
         <v>54206</v>
       </c>
       <c r="E43" t="s">
@@ -2261,13 +2269,13 @@
       <c r="A44" t="s">
         <v>48</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B44" s="1">
         <v>54</v>
       </c>
       <c r="C44" t="s">
         <v>49</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="3">
         <v>54245</v>
       </c>
       <c r="E44" t="s">
@@ -2278,13 +2286,13 @@
       <c r="A45" t="s">
         <v>48</v>
       </c>
-      <c r="B45" s="2">
+      <c r="B45" s="1">
         <v>54</v>
       </c>
       <c r="C45" t="s">
         <v>49</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="3">
         <v>54250</v>
       </c>
       <c r="E45" t="s">
@@ -2295,13 +2303,13 @@
       <c r="A46" t="s">
         <v>48</v>
       </c>
-      <c r="B46" s="2">
+      <c r="B46" s="1">
         <v>54</v>
       </c>
       <c r="C46" t="s">
         <v>49</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="3">
         <v>54344</v>
       </c>
       <c r="E46" t="s">
@@ -2312,13 +2320,13 @@
       <c r="A47" t="s">
         <v>48</v>
       </c>
-      <c r="B47" s="2">
+      <c r="B47" s="1">
         <v>54</v>
       </c>
       <c r="C47" t="s">
         <v>49</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="3">
         <v>54670</v>
       </c>
       <c r="E47" t="s">
@@ -2329,13 +2337,13 @@
       <c r="A48" t="s">
         <v>48</v>
       </c>
-      <c r="B48" s="2">
+      <c r="B48" s="1">
         <v>54</v>
       </c>
       <c r="C48" t="s">
         <v>49</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="3">
         <v>54720</v>
       </c>
       <c r="E48" t="s">
@@ -2346,13 +2354,13 @@
       <c r="A49" t="s">
         <v>48</v>
       </c>
-      <c r="B49" s="2">
+      <c r="B49" s="1">
         <v>54</v>
       </c>
       <c r="C49" t="s">
         <v>49</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="3">
         <v>54800</v>
       </c>
       <c r="E49" t="s">
@@ -2363,13 +2371,13 @@
       <c r="A50" t="s">
         <v>48</v>
       </c>
-      <c r="B50" s="2">
+      <c r="B50" s="1">
         <v>54</v>
       </c>
       <c r="C50" t="s">
         <v>49</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="3">
         <v>54810</v>
       </c>
       <c r="E50" t="s">
@@ -2380,13 +2388,13 @@
       <c r="A51" t="s">
         <v>58</v>
       </c>
-      <c r="B51" s="2">
+      <c r="B51" s="1">
         <v>5</v>
       </c>
       <c r="C51" t="s">
         <v>34</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51" s="3">
         <v>5475</v>
       </c>
       <c r="E51" t="s">
@@ -2397,13 +2405,13 @@
       <c r="A52" t="s">
         <v>58</v>
       </c>
-      <c r="B52" s="2">
+      <c r="B52" s="1">
         <v>5</v>
       </c>
       <c r="C52" t="s">
         <v>34</v>
       </c>
-      <c r="D52" s="1">
+      <c r="D52" s="3">
         <v>5873</v>
       </c>
       <c r="E52" t="s">
@@ -2414,13 +2422,13 @@
       <c r="A53" t="s">
         <v>58</v>
       </c>
-      <c r="B53" s="2">
+      <c r="B53" s="1">
         <v>27</v>
       </c>
       <c r="C53" t="s">
         <v>58</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53" s="3">
         <v>27006</v>
       </c>
       <c r="E53" t="s">
@@ -2431,13 +2439,13 @@
       <c r="A54" t="s">
         <v>58</v>
       </c>
-      <c r="B54" s="2">
+      <c r="B54" s="1">
         <v>27</v>
       </c>
       <c r="C54" t="s">
         <v>58</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54" s="3">
         <v>27099</v>
       </c>
       <c r="E54" t="s">
@@ -2448,13 +2456,13 @@
       <c r="A55" t="s">
         <v>58</v>
       </c>
-      <c r="B55" s="2">
+      <c r="B55" s="1">
         <v>27</v>
       </c>
       <c r="C55" t="s">
         <v>58</v>
       </c>
-      <c r="D55" s="1">
+      <c r="D55" s="3">
         <v>27150</v>
       </c>
       <c r="E55" t="s">
@@ -2465,13 +2473,13 @@
       <c r="A56" t="s">
         <v>58</v>
       </c>
-      <c r="B56" s="2">
+      <c r="B56" s="1">
         <v>27</v>
       </c>
       <c r="C56" t="s">
         <v>58</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="3">
         <v>27205</v>
       </c>
       <c r="E56" t="s">
@@ -2482,13 +2490,13 @@
       <c r="A57" t="s">
         <v>58</v>
       </c>
-      <c r="B57" s="2">
+      <c r="B57" s="1">
         <v>27</v>
       </c>
       <c r="C57" t="s">
         <v>58</v>
       </c>
-      <c r="D57" s="1">
+      <c r="D57" s="3">
         <v>27250</v>
       </c>
       <c r="E57" t="s">
@@ -2499,13 +2507,13 @@
       <c r="A58" t="s">
         <v>58</v>
       </c>
-      <c r="B58" s="2">
+      <c r="B58" s="1">
         <v>27</v>
       </c>
       <c r="C58" t="s">
         <v>58</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58" s="3">
         <v>27361</v>
       </c>
       <c r="E58" t="s">
@@ -2516,13 +2524,13 @@
       <c r="A59" t="s">
         <v>58</v>
       </c>
-      <c r="B59" s="2">
+      <c r="B59" s="1">
         <v>27</v>
       </c>
       <c r="C59" t="s">
         <v>58</v>
       </c>
-      <c r="D59" s="1">
+      <c r="D59" s="3">
         <v>27425</v>
       </c>
       <c r="E59" t="s">
@@ -2533,13 +2541,13 @@
       <c r="A60" t="s">
         <v>58</v>
       </c>
-      <c r="B60" s="2">
+      <c r="B60" s="1">
         <v>27</v>
       </c>
       <c r="C60" t="s">
         <v>58</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60" s="3">
         <v>27450</v>
       </c>
       <c r="E60" t="s">
@@ -2550,13 +2558,13 @@
       <c r="A61" t="s">
         <v>58</v>
       </c>
-      <c r="B61" s="2">
+      <c r="B61" s="1">
         <v>27</v>
       </c>
       <c r="C61" t="s">
         <v>58</v>
       </c>
-      <c r="D61" s="1">
+      <c r="D61" s="3">
         <v>27491</v>
       </c>
       <c r="E61" t="s">
@@ -2567,13 +2575,13 @@
       <c r="A62" t="s">
         <v>58</v>
       </c>
-      <c r="B62" s="2">
+      <c r="B62" s="1">
         <v>27</v>
       </c>
       <c r="C62" t="s">
         <v>58</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62" s="3">
         <v>27615</v>
       </c>
       <c r="E62" t="s">
@@ -2584,13 +2592,13 @@
       <c r="A63" t="s">
         <v>58</v>
       </c>
-      <c r="B63" s="2">
+      <c r="B63" s="1">
         <v>27</v>
       </c>
       <c r="C63" t="s">
         <v>58</v>
       </c>
-      <c r="D63" s="1">
+      <c r="D63" s="3">
         <v>27745</v>
       </c>
       <c r="E63" t="s">
@@ -2601,13 +2609,13 @@
       <c r="A64" t="s">
         <v>58</v>
       </c>
-      <c r="B64" s="2">
+      <c r="B64" s="1">
         <v>27</v>
       </c>
       <c r="C64" t="s">
         <v>58</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64" s="3">
         <v>27800</v>
       </c>
       <c r="E64" t="s">
@@ -2618,13 +2626,13 @@
       <c r="A65" t="s">
         <v>73</v>
       </c>
-      <c r="B65" s="2">
+      <c r="B65" s="1">
         <v>18</v>
       </c>
       <c r="C65" t="s">
         <v>74</v>
       </c>
-      <c r="D65" s="1">
+      <c r="D65" s="3">
         <v>18029</v>
       </c>
       <c r="E65" t="s">
@@ -2635,13 +2643,13 @@
       <c r="A66" t="s">
         <v>73</v>
       </c>
-      <c r="B66" s="2">
+      <c r="B66" s="1">
         <v>18</v>
       </c>
       <c r="C66" t="s">
         <v>74</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66" s="3">
         <v>18094</v>
       </c>
       <c r="E66" t="s">
@@ -2652,13 +2660,13 @@
       <c r="A67" t="s">
         <v>73</v>
       </c>
-      <c r="B67" s="2">
+      <c r="B67" s="1">
         <v>18</v>
       </c>
       <c r="C67" t="s">
         <v>74</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="3">
         <v>18150</v>
       </c>
       <c r="E67" t="s">
@@ -2669,13 +2677,13 @@
       <c r="A68" t="s">
         <v>73</v>
       </c>
-      <c r="B68" s="2">
+      <c r="B68" s="1">
         <v>18</v>
       </c>
       <c r="C68" t="s">
         <v>74</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="3">
         <v>18205</v>
       </c>
       <c r="E68" t="s">
@@ -2686,13 +2694,13 @@
       <c r="A69" t="s">
         <v>73</v>
       </c>
-      <c r="B69" s="2">
+      <c r="B69" s="1">
         <v>18</v>
       </c>
       <c r="C69" t="s">
         <v>74</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69" s="3">
         <v>18247</v>
       </c>
       <c r="E69" t="s">
@@ -2703,13 +2711,13 @@
       <c r="A70" t="s">
         <v>73</v>
       </c>
-      <c r="B70" s="2">
+      <c r="B70" s="1">
         <v>18</v>
       </c>
       <c r="C70" t="s">
         <v>74</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70" s="3">
         <v>18256</v>
       </c>
       <c r="E70" t="s">
@@ -2720,13 +2728,13 @@
       <c r="A71" t="s">
         <v>73</v>
       </c>
-      <c r="B71" s="2">
+      <c r="B71" s="1">
         <v>18</v>
       </c>
       <c r="C71" t="s">
         <v>74</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71" s="3">
         <v>18001</v>
       </c>
       <c r="E71" t="s">
@@ -2737,13 +2745,13 @@
       <c r="A72" t="s">
         <v>73</v>
       </c>
-      <c r="B72" s="2">
+      <c r="B72" s="1">
         <v>18</v>
       </c>
       <c r="C72" t="s">
         <v>74</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72" s="3">
         <v>18410</v>
       </c>
       <c r="E72" t="s">
@@ -2754,13 +2762,13 @@
       <c r="A73" t="s">
         <v>73</v>
       </c>
-      <c r="B73" s="2">
+      <c r="B73" s="1">
         <v>18</v>
       </c>
       <c r="C73" t="s">
         <v>74</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73" s="3">
         <v>18460</v>
       </c>
       <c r="E73" t="s">
@@ -2771,13 +2779,13 @@
       <c r="A74" t="s">
         <v>73</v>
       </c>
-      <c r="B74" s="2">
+      <c r="B74" s="1">
         <v>18</v>
       </c>
       <c r="C74" t="s">
         <v>74</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D74" s="3">
         <v>18479</v>
       </c>
       <c r="E74" t="s">
@@ -2788,13 +2796,13 @@
       <c r="A75" t="s">
         <v>73</v>
       </c>
-      <c r="B75" s="2">
+      <c r="B75" s="1">
         <v>18</v>
       </c>
       <c r="C75" t="s">
         <v>74</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D75" s="3">
         <v>18592</v>
       </c>
       <c r="E75" t="s">
@@ -2805,13 +2813,13 @@
       <c r="A76" t="s">
         <v>73</v>
       </c>
-      <c r="B76" s="2">
+      <c r="B76" s="1">
         <v>18</v>
       </c>
       <c r="C76" t="s">
         <v>74</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76" s="3">
         <v>18610</v>
       </c>
       <c r="E76" t="s">
@@ -2822,13 +2830,13 @@
       <c r="A77" t="s">
         <v>73</v>
       </c>
-      <c r="B77" s="2">
+      <c r="B77" s="1">
         <v>18</v>
       </c>
       <c r="C77" t="s">
         <v>74</v>
       </c>
-      <c r="D77" s="1">
+      <c r="D77" s="3">
         <v>18753</v>
       </c>
       <c r="E77" t="s">
@@ -2839,13 +2847,13 @@
       <c r="A78" t="s">
         <v>73</v>
       </c>
-      <c r="B78" s="2">
+      <c r="B78" s="1">
         <v>18</v>
       </c>
       <c r="C78" t="s">
         <v>74</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D78" s="3">
         <v>18756</v>
       </c>
       <c r="E78" t="s">
@@ -2856,13 +2864,13 @@
       <c r="A79" t="s">
         <v>73</v>
       </c>
-      <c r="B79" s="2">
+      <c r="B79" s="1">
         <v>18</v>
       </c>
       <c r="C79" t="s">
         <v>74</v>
       </c>
-      <c r="D79" s="1">
+      <c r="D79" s="3">
         <v>18785</v>
       </c>
       <c r="E79" t="s">
@@ -2873,13 +2881,13 @@
       <c r="A80" t="s">
         <v>73</v>
       </c>
-      <c r="B80" s="2">
+      <c r="B80" s="1">
         <v>18</v>
       </c>
       <c r="C80" t="s">
         <v>74</v>
       </c>
-      <c r="D80" s="1">
+      <c r="D80" s="3">
         <v>18860</v>
       </c>
       <c r="E80" t="s">
@@ -2890,13 +2898,13 @@
       <c r="A81" t="s">
         <v>73</v>
       </c>
-      <c r="B81" s="2">
+      <c r="B81" s="1">
         <v>41</v>
       </c>
       <c r="C81" t="s">
         <v>91</v>
       </c>
-      <c r="D81" s="1">
+      <c r="D81" s="3">
         <v>41020</v>
       </c>
       <c r="E81" t="s">
@@ -2907,13 +2915,13 @@
       <c r="A82" t="s">
         <v>93</v>
       </c>
-      <c r="B82" s="2">
+      <c r="B82" s="1">
         <v>95</v>
       </c>
       <c r="C82" t="s">
         <v>94</v>
       </c>
-      <c r="D82" s="1">
+      <c r="D82" s="3">
         <v>95015</v>
       </c>
       <c r="E82" t="s">
@@ -2924,13 +2932,13 @@
       <c r="A83" t="s">
         <v>93</v>
       </c>
-      <c r="B83" s="2">
+      <c r="B83" s="1">
         <v>95</v>
       </c>
       <c r="C83" t="s">
         <v>94</v>
       </c>
-      <c r="D83" s="1">
+      <c r="D83" s="3">
         <v>95025</v>
       </c>
       <c r="E83" t="s">
@@ -2941,13 +2949,13 @@
       <c r="A84" t="s">
         <v>93</v>
       </c>
-      <c r="B84" s="2">
+      <c r="B84" s="1">
         <v>95</v>
       </c>
       <c r="C84" t="s">
         <v>94</v>
       </c>
-      <c r="D84" s="1">
+      <c r="D84" s="3">
         <v>95200</v>
       </c>
       <c r="E84" t="s">
@@ -2958,13 +2966,13 @@
       <c r="A85" t="s">
         <v>93</v>
       </c>
-      <c r="B85" s="2">
+      <c r="B85" s="1">
         <v>95</v>
       </c>
       <c r="C85" t="s">
         <v>94</v>
       </c>
-      <c r="D85" s="1">
+      <c r="D85" s="3">
         <v>95001</v>
       </c>
       <c r="E85" t="s">
@@ -2975,13 +2983,13 @@
       <c r="A86" t="s">
         <v>93</v>
       </c>
-      <c r="B86" s="2">
+      <c r="B86" s="1">
         <v>50</v>
       </c>
       <c r="C86" t="s">
         <v>99</v>
       </c>
-      <c r="D86" s="1">
+      <c r="D86" s="3">
         <v>50350</v>
       </c>
       <c r="E86" t="s">
@@ -2992,13 +3000,13 @@
       <c r="A87" t="s">
         <v>93</v>
       </c>
-      <c r="B87" s="2">
+      <c r="B87" s="1">
         <v>50</v>
       </c>
       <c r="C87" t="s">
         <v>99</v>
       </c>
-      <c r="D87" s="1">
+      <c r="D87" s="3">
         <v>50325</v>
       </c>
       <c r="E87" t="s">
@@ -3009,13 +3017,13 @@
       <c r="A88" t="s">
         <v>93</v>
       </c>
-      <c r="B88" s="2">
+      <c r="B88" s="1">
         <v>50</v>
       </c>
       <c r="C88" t="s">
         <v>99</v>
       </c>
-      <c r="D88" s="1">
+      <c r="D88" s="3">
         <v>50330</v>
       </c>
       <c r="E88" t="s">
@@ -3026,13 +3034,13 @@
       <c r="A89" t="s">
         <v>93</v>
       </c>
-      <c r="B89" s="2">
+      <c r="B89" s="1">
         <v>50</v>
       </c>
       <c r="C89" t="s">
         <v>99</v>
       </c>
-      <c r="D89" s="1">
+      <c r="D89" s="3">
         <v>50450</v>
       </c>
       <c r="E89" t="s">
@@ -3043,13 +3051,13 @@
       <c r="A90" t="s">
         <v>93</v>
       </c>
-      <c r="B90" s="2">
+      <c r="B90" s="1">
         <v>50</v>
       </c>
       <c r="C90" t="s">
         <v>99</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90" s="3">
         <v>50577</v>
       </c>
       <c r="E90" t="s">
@@ -3060,13 +3068,13 @@
       <c r="A91" t="s">
         <v>93</v>
       </c>
-      <c r="B91" s="2">
+      <c r="B91" s="1">
         <v>50</v>
       </c>
       <c r="C91" t="s">
         <v>99</v>
       </c>
-      <c r="D91" s="1">
+      <c r="D91" s="3">
         <v>50590</v>
       </c>
       <c r="E91" t="s">
@@ -3077,13 +3085,13 @@
       <c r="A92" t="s">
         <v>93</v>
       </c>
-      <c r="B92" s="2">
+      <c r="B92" s="1">
         <v>50</v>
       </c>
       <c r="C92" t="s">
         <v>99</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D92" s="3">
         <v>50370</v>
       </c>
       <c r="E92" t="s">
@@ -3094,13 +3102,13 @@
       <c r="A93" t="s">
         <v>93</v>
       </c>
-      <c r="B93" s="2">
+      <c r="B93" s="1">
         <v>50</v>
       </c>
       <c r="C93" t="s">
         <v>99</v>
       </c>
-      <c r="D93" s="1">
+      <c r="D93" s="3">
         <v>50711</v>
       </c>
       <c r="E93" t="s">
@@ -3111,13 +3119,13 @@
       <c r="A94" t="s">
         <v>107</v>
       </c>
-      <c r="B94" s="2">
+      <c r="B94" s="1">
         <v>13</v>
       </c>
       <c r="C94" t="s">
         <v>108</v>
       </c>
-      <c r="D94" s="1">
+      <c r="D94" s="3">
         <v>13212</v>
       </c>
       <c r="E94" t="s">
@@ -3128,13 +3136,13 @@
       <c r="A95" t="s">
         <v>107</v>
       </c>
-      <c r="B95" s="2">
+      <c r="B95" s="1">
         <v>13</v>
       </c>
       <c r="C95" t="s">
         <v>108</v>
       </c>
-      <c r="D95" s="1">
+      <c r="D95" s="3">
         <v>13244</v>
       </c>
       <c r="E95" t="s">
@@ -3145,13 +3153,13 @@
       <c r="A96" t="s">
         <v>107</v>
       </c>
-      <c r="B96" s="2">
+      <c r="B96" s="1">
         <v>13</v>
       </c>
       <c r="C96" t="s">
         <v>108</v>
       </c>
-      <c r="D96" s="1">
+      <c r="D96" s="3">
         <v>13248</v>
       </c>
       <c r="E96" t="s">
@@ -3162,13 +3170,13 @@
       <c r="A97" t="s">
         <v>107</v>
       </c>
-      <c r="B97" s="2">
+      <c r="B97" s="1">
         <v>13</v>
       </c>
       <c r="C97" t="s">
         <v>108</v>
       </c>
-      <c r="D97" s="1">
+      <c r="D97" s="3">
         <v>13442</v>
       </c>
       <c r="E97" t="s">
@@ -3179,13 +3187,13 @@
       <c r="A98" t="s">
         <v>107</v>
       </c>
-      <c r="B98" s="2">
+      <c r="B98" s="1">
         <v>13</v>
       </c>
       <c r="C98" t="s">
         <v>108</v>
       </c>
-      <c r="D98" s="1">
+      <c r="D98" s="3">
         <v>13654</v>
       </c>
       <c r="E98" t="s">
@@ -3196,13 +3204,13 @@
       <c r="A99" t="s">
         <v>107</v>
       </c>
-      <c r="B99" s="2">
+      <c r="B99" s="1">
         <v>13</v>
       </c>
       <c r="C99" t="s">
         <v>108</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99" s="3">
         <v>13657</v>
       </c>
       <c r="E99" t="s">
@@ -3213,13 +3221,13 @@
       <c r="A100" t="s">
         <v>107</v>
       </c>
-      <c r="B100" s="2">
+      <c r="B100" s="1">
         <v>13</v>
       </c>
       <c r="C100" t="s">
         <v>108</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100" s="3">
         <v>13894</v>
       </c>
       <c r="E100" t="s">
@@ -3230,13 +3238,13 @@
       <c r="A101" t="s">
         <v>107</v>
       </c>
-      <c r="B101" s="2">
+      <c r="B101" s="1">
         <v>70</v>
       </c>
       <c r="C101" t="s">
         <v>116</v>
       </c>
-      <c r="D101" s="1">
+      <c r="D101" s="3">
         <v>70230</v>
       </c>
       <c r="E101" t="s">
@@ -3247,13 +3255,13 @@
       <c r="A102" t="s">
         <v>107</v>
       </c>
-      <c r="B102" s="2">
+      <c r="B102" s="1">
         <v>70</v>
       </c>
       <c r="C102" t="s">
         <v>116</v>
       </c>
-      <c r="D102" s="1">
+      <c r="D102" s="3">
         <v>70204</v>
       </c>
       <c r="E102" t="s">
@@ -3264,13 +3272,13 @@
       <c r="A103" t="s">
         <v>107</v>
       </c>
-      <c r="B103" s="2">
+      <c r="B103" s="1">
         <v>70</v>
       </c>
       <c r="C103" t="s">
         <v>116</v>
       </c>
-      <c r="D103" s="1">
+      <c r="D103" s="3">
         <v>70418</v>
       </c>
       <c r="E103" t="s">
@@ -3281,13 +3289,13 @@
       <c r="A104" t="s">
         <v>107</v>
       </c>
-      <c r="B104" s="2">
+      <c r="B104" s="1">
         <v>70</v>
       </c>
       <c r="C104" t="s">
         <v>116</v>
       </c>
-      <c r="D104" s="1">
+      <c r="D104" s="3">
         <v>70473</v>
       </c>
       <c r="E104" t="s">
@@ -3298,13 +3306,13 @@
       <c r="A105" t="s">
         <v>107</v>
       </c>
-      <c r="B105" s="2">
+      <c r="B105" s="1">
         <v>70</v>
       </c>
       <c r="C105" t="s">
         <v>116</v>
       </c>
-      <c r="D105" s="1">
+      <c r="D105" s="3">
         <v>70508</v>
       </c>
       <c r="E105" t="s">
@@ -3315,13 +3323,13 @@
       <c r="A106" t="s">
         <v>107</v>
       </c>
-      <c r="B106" s="2">
+      <c r="B106" s="1">
         <v>70</v>
       </c>
       <c r="C106" t="s">
         <v>116</v>
       </c>
-      <c r="D106" s="1">
+      <c r="D106" s="3">
         <v>70523</v>
       </c>
       <c r="E106" t="s">
@@ -3332,13 +3340,13 @@
       <c r="A107" t="s">
         <v>107</v>
       </c>
-      <c r="B107" s="2">
+      <c r="B107" s="1">
         <v>70</v>
       </c>
       <c r="C107" t="s">
         <v>116</v>
       </c>
-      <c r="D107" s="1">
+      <c r="D107" s="3">
         <v>70713</v>
       </c>
       <c r="E107" t="s">
@@ -3349,13 +3357,13 @@
       <c r="A108" t="s">
         <v>107</v>
       </c>
-      <c r="B108" s="2">
+      <c r="B108" s="1">
         <v>70</v>
       </c>
       <c r="C108" t="s">
         <v>116</v>
       </c>
-      <c r="D108" s="1">
+      <c r="D108" s="3">
         <v>70823</v>
       </c>
       <c r="E108" t="s">
@@ -3366,13 +3374,13 @@
       <c r="A109" t="s">
         <v>125</v>
       </c>
-      <c r="B109" s="2">
+      <c r="B109" s="1">
         <v>19</v>
       </c>
       <c r="C109" t="s">
         <v>1</v>
       </c>
-      <c r="D109" s="1">
+      <c r="D109" s="3">
         <v>19318</v>
       </c>
       <c r="E109" t="s">
@@ -3383,13 +3391,13 @@
       <c r="A110" t="s">
         <v>125</v>
       </c>
-      <c r="B110" s="2">
+      <c r="B110" s="1">
         <v>19</v>
       </c>
       <c r="C110" t="s">
         <v>1</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D110" s="3">
         <v>19418</v>
       </c>
       <c r="E110" t="s">
@@ -3400,13 +3408,13 @@
       <c r="A111" t="s">
         <v>125</v>
       </c>
-      <c r="B111" s="2">
+      <c r="B111" s="1">
         <v>19</v>
       </c>
       <c r="C111" t="s">
         <v>1</v>
       </c>
-      <c r="D111" s="1">
+      <c r="D111" s="3">
         <v>19809</v>
       </c>
       <c r="E111" t="s">
@@ -3417,13 +3425,13 @@
       <c r="A112" t="s">
         <v>125</v>
       </c>
-      <c r="B112" s="2">
+      <c r="B112" s="1">
         <v>76</v>
       </c>
       <c r="C112" t="s">
         <v>25</v>
       </c>
-      <c r="D112" s="1">
+      <c r="D112" s="3">
         <v>76109</v>
       </c>
       <c r="E112" t="s">
@@ -3434,13 +3442,13 @@
       <c r="A113" t="s">
         <v>130</v>
       </c>
-      <c r="B113" s="2">
+      <c r="B113" s="1">
         <v>52</v>
       </c>
       <c r="C113" t="s">
         <v>19</v>
       </c>
-      <c r="D113" s="1">
+      <c r="D113" s="3">
         <v>52079</v>
       </c>
       <c r="E113" t="s">
@@ -3451,13 +3459,13 @@
       <c r="A114" t="s">
         <v>130</v>
       </c>
-      <c r="B114" s="2">
+      <c r="B114" s="1">
         <v>52</v>
       </c>
       <c r="C114" t="s">
         <v>19</v>
       </c>
-      <c r="D114" s="1">
+      <c r="D114" s="3">
         <v>52250</v>
       </c>
       <c r="E114" t="s">
@@ -3468,13 +3476,13 @@
       <c r="A115" t="s">
         <v>130</v>
       </c>
-      <c r="B115" s="2">
+      <c r="B115" s="1">
         <v>52</v>
       </c>
       <c r="C115" t="s">
         <v>19</v>
       </c>
-      <c r="D115" s="1">
+      <c r="D115" s="3">
         <v>52520</v>
       </c>
       <c r="E115" t="s">
@@ -3485,13 +3493,13 @@
       <c r="A116" t="s">
         <v>130</v>
       </c>
-      <c r="B116" s="2">
+      <c r="B116" s="1">
         <v>52</v>
       </c>
       <c r="C116" t="s">
         <v>19</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116" s="3">
         <v>52390</v>
       </c>
       <c r="E116" t="s">
@@ -3502,13 +3510,13 @@
       <c r="A117" t="s">
         <v>130</v>
       </c>
-      <c r="B117" s="2">
+      <c r="B117" s="1">
         <v>52</v>
       </c>
       <c r="C117" t="s">
         <v>19</v>
       </c>
-      <c r="D117" s="1">
+      <c r="D117" s="3">
         <v>52427</v>
       </c>
       <c r="E117" t="s">
@@ -3519,13 +3527,13 @@
       <c r="A118" t="s">
         <v>130</v>
       </c>
-      <c r="B118" s="2">
+      <c r="B118" s="1">
         <v>52</v>
       </c>
       <c r="C118" t="s">
         <v>19</v>
       </c>
-      <c r="D118" s="1">
+      <c r="D118" s="3">
         <v>52473</v>
       </c>
       <c r="E118" t="s">
@@ -3536,13 +3544,13 @@
       <c r="A119" t="s">
         <v>130</v>
       </c>
-      <c r="B119" s="2">
+      <c r="B119" s="1">
         <v>52</v>
       </c>
       <c r="C119" t="s">
         <v>19</v>
       </c>
-      <c r="D119" s="1">
+      <c r="D119" s="3">
         <v>52490</v>
       </c>
       <c r="E119" t="s">
@@ -3553,13 +3561,13 @@
       <c r="A120" t="s">
         <v>130</v>
       </c>
-      <c r="B120" s="2">
+      <c r="B120" s="1">
         <v>52</v>
       </c>
       <c r="C120" t="s">
         <v>19</v>
       </c>
-      <c r="D120" s="1">
+      <c r="D120" s="3">
         <v>52612</v>
       </c>
       <c r="E120" t="s">
@@ -3570,13 +3578,13 @@
       <c r="A121" t="s">
         <v>130</v>
       </c>
-      <c r="B121" s="2">
+      <c r="B121" s="1">
         <v>52</v>
       </c>
       <c r="C121" t="s">
         <v>19</v>
       </c>
-      <c r="D121" s="1">
+      <c r="D121" s="3">
         <v>52621</v>
       </c>
       <c r="E121" t="s">
@@ -3587,13 +3595,13 @@
       <c r="A122" t="s">
         <v>130</v>
       </c>
-      <c r="B122" s="2">
+      <c r="B122" s="1">
         <v>52</v>
       </c>
       <c r="C122" t="s">
         <v>19</v>
       </c>
-      <c r="D122" s="1">
+      <c r="D122" s="3">
         <v>52835</v>
       </c>
       <c r="E122" t="s">
@@ -3604,13 +3612,13 @@
       <c r="A123" t="s">
         <v>130</v>
       </c>
-      <c r="B123" s="2">
+      <c r="B123" s="1">
         <v>52</v>
       </c>
       <c r="C123" t="s">
         <v>19</v>
       </c>
-      <c r="D123" s="1">
+      <c r="D123" s="3">
         <v>52696</v>
       </c>
       <c r="E123" t="s">
@@ -3621,13 +3629,13 @@
       <c r="A124" t="s">
         <v>142</v>
       </c>
-      <c r="B124" s="2">
+      <c r="B124" s="1">
         <v>86</v>
       </c>
       <c r="C124" t="s">
         <v>142</v>
       </c>
-      <c r="D124" s="1">
+      <c r="D124" s="3">
         <v>86573</v>
       </c>
       <c r="E124" t="s">
@@ -3638,13 +3646,13 @@
       <c r="A125" t="s">
         <v>142</v>
       </c>
-      <c r="B125" s="2">
+      <c r="B125" s="1">
         <v>86</v>
       </c>
       <c r="C125" t="s">
         <v>142</v>
       </c>
-      <c r="D125" s="1">
+      <c r="D125" s="3">
         <v>86001</v>
       </c>
       <c r="E125" t="s">
@@ -3655,13 +3663,13 @@
       <c r="A126" t="s">
         <v>142</v>
       </c>
-      <c r="B126" s="2">
+      <c r="B126" s="1">
         <v>86</v>
       </c>
       <c r="C126" t="s">
         <v>142</v>
       </c>
-      <c r="D126" s="1">
+      <c r="D126" s="3">
         <v>86320</v>
       </c>
       <c r="E126" t="s">
@@ -3672,13 +3680,13 @@
       <c r="A127" t="s">
         <v>142</v>
       </c>
-      <c r="B127" s="2">
+      <c r="B127" s="1">
         <v>86</v>
       </c>
       <c r="C127" t="s">
         <v>142</v>
       </c>
-      <c r="D127" s="1">
+      <c r="D127" s="3">
         <v>86568</v>
       </c>
       <c r="E127" t="s">
@@ -3689,13 +3697,13 @@
       <c r="A128" t="s">
         <v>142</v>
       </c>
-      <c r="B128" s="2">
+      <c r="B128" s="1">
         <v>86</v>
       </c>
       <c r="C128" t="s">
         <v>142</v>
       </c>
-      <c r="D128" s="1">
+      <c r="D128" s="3">
         <v>86569</v>
       </c>
       <c r="E128" t="s">
@@ -3706,13 +3714,13 @@
       <c r="A129" t="s">
         <v>142</v>
       </c>
-      <c r="B129" s="2">
+      <c r="B129" s="1">
         <v>86</v>
       </c>
       <c r="C129" t="s">
         <v>142</v>
       </c>
-      <c r="D129" s="1">
+      <c r="D129" s="3">
         <v>86571</v>
       </c>
       <c r="E129" t="s">
@@ -3723,13 +3731,13 @@
       <c r="A130" t="s">
         <v>142</v>
       </c>
-      <c r="B130" s="2">
+      <c r="B130" s="1">
         <v>86</v>
       </c>
       <c r="C130" t="s">
         <v>142</v>
       </c>
-      <c r="D130" s="1">
+      <c r="D130" s="3">
         <v>86757</v>
       </c>
       <c r="E130" t="s">
@@ -3740,13 +3748,13 @@
       <c r="A131" t="s">
         <v>142</v>
       </c>
-      <c r="B131" s="2">
+      <c r="B131" s="1">
         <v>86</v>
       </c>
       <c r="C131" t="s">
         <v>142</v>
       </c>
-      <c r="D131" s="1">
+      <c r="D131" s="3">
         <v>86865</v>
       </c>
       <c r="E131" t="s">
@@ -3757,13 +3765,13 @@
       <c r="A132" t="s">
         <v>142</v>
       </c>
-      <c r="B132" s="2">
+      <c r="B132" s="1">
         <v>86</v>
       </c>
       <c r="C132" t="s">
         <v>142</v>
       </c>
-      <c r="D132" s="1">
+      <c r="D132" s="3">
         <v>86885</v>
       </c>
       <c r="E132" t="s">
@@ -3774,13 +3782,13 @@
       <c r="A133" t="s">
         <v>152</v>
       </c>
-      <c r="B133" s="2">
+      <c r="B133" s="1">
         <v>20</v>
       </c>
       <c r="C133" t="s">
         <v>153</v>
       </c>
-      <c r="D133" s="1">
+      <c r="D133" s="3">
         <v>20013</v>
       </c>
       <c r="E133" t="s">
@@ -3791,13 +3799,13 @@
       <c r="A134" t="s">
         <v>152</v>
       </c>
-      <c r="B134" s="2">
+      <c r="B134" s="1">
         <v>20</v>
       </c>
       <c r="C134" t="s">
         <v>153</v>
       </c>
-      <c r="D134" s="1">
+      <c r="D134" s="3">
         <v>20045</v>
       </c>
       <c r="E134" t="s">
@@ -3808,13 +3816,13 @@
       <c r="A135" t="s">
         <v>152</v>
       </c>
-      <c r="B135" s="2">
+      <c r="B135" s="1">
         <v>20</v>
       </c>
       <c r="C135" t="s">
         <v>153</v>
       </c>
-      <c r="D135" s="1">
+      <c r="D135" s="3">
         <v>20400</v>
       </c>
       <c r="E135" t="s">
@@ -3825,13 +3833,13 @@
       <c r="A136" t="s">
         <v>152</v>
       </c>
-      <c r="B136" s="2">
+      <c r="B136" s="1">
         <v>20</v>
       </c>
       <c r="C136" t="s">
         <v>153</v>
       </c>
-      <c r="D136" s="1">
+      <c r="D136" s="3">
         <v>20621</v>
       </c>
       <c r="E136" t="s">
@@ -3842,13 +3850,13 @@
       <c r="A137" t="s">
         <v>152</v>
       </c>
-      <c r="B137" s="2">
+      <c r="B137" s="1">
         <v>20</v>
       </c>
       <c r="C137" t="s">
         <v>153</v>
       </c>
-      <c r="D137" s="1">
+      <c r="D137" s="3">
         <v>20443</v>
       </c>
       <c r="E137" t="s">
@@ -3859,13 +3867,13 @@
       <c r="A138" t="s">
         <v>152</v>
       </c>
-      <c r="B138" s="2">
+      <c r="B138" s="1">
         <v>20</v>
       </c>
       <c r="C138" t="s">
         <v>153</v>
       </c>
-      <c r="D138" s="1">
+      <c r="D138" s="3">
         <v>20570</v>
       </c>
       <c r="E138" t="s">
@@ -3876,13 +3884,13 @@
       <c r="A139" t="s">
         <v>152</v>
       </c>
-      <c r="B139" s="2">
+      <c r="B139" s="1">
         <v>20</v>
       </c>
       <c r="C139" t="s">
         <v>153</v>
       </c>
-      <c r="D139" s="1">
+      <c r="D139" s="3">
         <v>20750</v>
       </c>
       <c r="E139" t="s">
@@ -3893,13 +3901,13 @@
       <c r="A140" t="s">
         <v>152</v>
       </c>
-      <c r="B140" s="2">
+      <c r="B140" s="1">
         <v>20</v>
       </c>
       <c r="C140" t="s">
         <v>153</v>
       </c>
-      <c r="D140" s="1">
+      <c r="D140" s="3">
         <v>20001</v>
       </c>
       <c r="E140" t="s">
@@ -3910,13 +3918,13 @@
       <c r="A141" t="s">
         <v>152</v>
       </c>
-      <c r="B141" s="2">
+      <c r="B141" s="1">
         <v>44</v>
       </c>
       <c r="C141" t="s">
         <v>162</v>
       </c>
-      <c r="D141" s="1">
+      <c r="D141" s="3">
         <v>44090</v>
       </c>
       <c r="E141" t="s">
@@ -3927,13 +3935,13 @@
       <c r="A142" t="s">
         <v>152</v>
       </c>
-      <c r="B142" s="2">
+      <c r="B142" s="1">
         <v>44</v>
       </c>
       <c r="C142" t="s">
         <v>162</v>
       </c>
-      <c r="D142" s="1">
+      <c r="D142" s="3">
         <v>44279</v>
       </c>
       <c r="E142" t="s">
@@ -3944,13 +3952,13 @@
       <c r="A143" t="s">
         <v>152</v>
       </c>
-      <c r="B143" s="2">
+      <c r="B143" s="1">
         <v>44</v>
       </c>
       <c r="C143" t="s">
         <v>162</v>
       </c>
-      <c r="D143" s="1">
+      <c r="D143" s="3">
         <v>44650</v>
       </c>
       <c r="E143" t="s">
@@ -3961,13 +3969,13 @@
       <c r="A144" t="s">
         <v>152</v>
       </c>
-      <c r="B144" s="2">
+      <c r="B144" s="1">
         <v>47</v>
       </c>
       <c r="C144" t="s">
         <v>166</v>
       </c>
-      <c r="D144" s="1">
+      <c r="D144" s="3">
         <v>47053</v>
       </c>
       <c r="E144" t="s">
@@ -3978,13 +3986,13 @@
       <c r="A145" t="s">
         <v>152</v>
       </c>
-      <c r="B145" s="2">
+      <c r="B145" s="1">
         <v>47</v>
       </c>
       <c r="C145" t="s">
         <v>166</v>
       </c>
-      <c r="D145" s="1">
+      <c r="D145" s="3">
         <v>47189</v>
       </c>
       <c r="E145" t="s">
@@ -3995,13 +4003,13 @@
       <c r="A146" t="s">
         <v>152</v>
       </c>
-      <c r="B146" s="2">
+      <c r="B146" s="1">
         <v>47</v>
       </c>
       <c r="C146" t="s">
         <v>166</v>
       </c>
-      <c r="D146" s="1">
+      <c r="D146" s="3">
         <v>47288</v>
       </c>
       <c r="E146" t="s">
@@ -4012,13 +4020,13 @@
       <c r="A147" t="s">
         <v>152</v>
       </c>
-      <c r="B147" s="2">
+      <c r="B147" s="1">
         <v>47</v>
       </c>
       <c r="C147" t="s">
         <v>166</v>
       </c>
-      <c r="D147" s="1">
+      <c r="D147" s="3">
         <v>47001</v>
       </c>
       <c r="E147" t="s">
@@ -4029,13 +4037,13 @@
       <c r="A148" t="s">
         <v>171</v>
       </c>
-      <c r="B148" s="2">
+      <c r="B148" s="1">
         <v>5</v>
       </c>
       <c r="C148" t="s">
         <v>34</v>
       </c>
-      <c r="D148" s="1">
+      <c r="D148" s="3">
         <v>5893</v>
       </c>
       <c r="E148" t="s">
@@ -4046,13 +4054,13 @@
       <c r="A149" t="s">
         <v>171</v>
       </c>
-      <c r="B149" s="2">
+      <c r="B149" s="1">
         <v>13</v>
       </c>
       <c r="C149" t="s">
         <v>108</v>
       </c>
-      <c r="D149" s="1">
+      <c r="D149" s="3">
         <v>13042</v>
       </c>
       <c r="E149" t="s">
@@ -4063,13 +4071,13 @@
       <c r="A150" t="s">
         <v>171</v>
       </c>
-      <c r="B150" s="2">
+      <c r="B150" s="1">
         <v>13</v>
       </c>
       <c r="C150" t="s">
         <v>108</v>
       </c>
-      <c r="D150" s="1">
+      <c r="D150" s="3">
         <v>13160</v>
       </c>
       <c r="E150" t="s">
@@ -4080,13 +4088,13 @@
       <c r="A151" t="s">
         <v>171</v>
       </c>
-      <c r="B151" s="2">
+      <c r="B151" s="1">
         <v>13</v>
       </c>
       <c r="C151" t="s">
         <v>108</v>
       </c>
-      <c r="D151" s="1">
+      <c r="D151" s="3">
         <v>13473</v>
       </c>
       <c r="E151" t="s">
@@ -4097,13 +4105,13 @@
       <c r="A152" t="s">
         <v>171</v>
       </c>
-      <c r="B152" s="2">
+      <c r="B152" s="1">
         <v>13</v>
       </c>
       <c r="C152" t="s">
         <v>108</v>
       </c>
-      <c r="D152" s="1">
+      <c r="D152" s="3">
         <v>13670</v>
       </c>
       <c r="E152" t="s">
@@ -4114,13 +4122,13 @@
       <c r="A153" t="s">
         <v>171</v>
       </c>
-      <c r="B153" s="2">
+      <c r="B153" s="1">
         <v>13</v>
       </c>
       <c r="C153" t="s">
         <v>108</v>
       </c>
-      <c r="D153" s="1">
+      <c r="D153" s="3">
         <v>13688</v>
       </c>
       <c r="E153" t="s">
@@ -4131,13 +4139,13 @@
       <c r="A154" t="s">
         <v>171</v>
       </c>
-      <c r="B154" s="2">
+      <c r="B154" s="1">
         <v>13</v>
       </c>
       <c r="C154" t="s">
         <v>108</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D154" s="3">
         <v>13744</v>
       </c>
       <c r="E154" t="s">
@@ -4148,13 +4156,13 @@
       <c r="A155" t="s">
         <v>178</v>
       </c>
-      <c r="B155" s="2">
+      <c r="B155" s="1">
         <v>23</v>
       </c>
       <c r="C155" t="s">
         <v>109</v>
       </c>
-      <c r="D155" s="1">
+      <c r="D155" s="3">
         <v>23466</v>
       </c>
       <c r="E155" t="s">
@@ -4165,13 +4173,13 @@
       <c r="A156" t="s">
         <v>178</v>
       </c>
-      <c r="B156" s="2">
+      <c r="B156" s="1">
         <v>23</v>
       </c>
       <c r="C156" t="s">
         <v>109</v>
       </c>
-      <c r="D156" s="1">
+      <c r="D156" s="3">
         <v>23580</v>
       </c>
       <c r="E156" t="s">
@@ -4182,13 +4190,13 @@
       <c r="A157" t="s">
         <v>178</v>
       </c>
-      <c r="B157" s="2">
+      <c r="B157" s="1">
         <v>23</v>
       </c>
       <c r="C157" t="s">
         <v>109</v>
       </c>
-      <c r="D157" s="1">
+      <c r="D157" s="3">
         <v>23682</v>
       </c>
       <c r="E157" t="s">
@@ -4199,13 +4207,13 @@
       <c r="A158" t="s">
         <v>178</v>
       </c>
-      <c r="B158" s="2">
+      <c r="B158" s="1">
         <v>23</v>
       </c>
       <c r="C158" t="s">
         <v>109</v>
       </c>
-      <c r="D158" s="1">
+      <c r="D158" s="3">
         <v>23807</v>
       </c>
       <c r="E158" t="s">
@@ -4216,13 +4224,13 @@
       <c r="A159" t="s">
         <v>178</v>
       </c>
-      <c r="B159" s="2">
+      <c r="B159" s="1">
         <v>23</v>
       </c>
       <c r="C159" t="s">
         <v>109</v>
       </c>
-      <c r="D159" s="1">
+      <c r="D159" s="3">
         <v>23855</v>
       </c>
       <c r="E159" t="s">
@@ -4233,13 +4241,13 @@
       <c r="A160" t="s">
         <v>184</v>
       </c>
-      <c r="B160" s="2">
+      <c r="B160" s="1">
         <v>73</v>
       </c>
       <c r="C160" t="s">
         <v>185</v>
       </c>
-      <c r="D160" s="1">
+      <c r="D160" s="3">
         <v>73067</v>
       </c>
       <c r="E160" t="s">
@@ -4250,13 +4258,13 @@
       <c r="A161" t="s">
         <v>184</v>
       </c>
-      <c r="B161" s="2">
+      <c r="B161" s="1">
         <v>73</v>
       </c>
       <c r="C161" t="s">
         <v>185</v>
       </c>
-      <c r="D161" s="1">
+      <c r="D161" s="3">
         <v>73168</v>
       </c>
       <c r="E161" t="s">
@@ -4267,13 +4275,13 @@
       <c r="A162" t="s">
         <v>184</v>
       </c>
-      <c r="B162" s="2">
+      <c r="B162" s="1">
         <v>73</v>
       </c>
       <c r="C162" t="s">
         <v>185</v>
       </c>
-      <c r="D162" s="1">
+      <c r="D162" s="3">
         <v>73555</v>
       </c>
       <c r="E162" t="s">
@@ -4284,13 +4292,13 @@
       <c r="A163" t="s">
         <v>184</v>
       </c>
-      <c r="B163" s="2">
+      <c r="B163" s="1">
         <v>73</v>
       </c>
       <c r="C163" t="s">
         <v>185</v>
       </c>
-      <c r="D163" s="1">
+      <c r="D163" s="3">
         <v>73616</v>
       </c>
       <c r="E163" t="s">
@@ -4301,13 +4309,13 @@
       <c r="A164" t="s">
         <v>190</v>
       </c>
-      <c r="B164" s="2">
+      <c r="B164" s="1">
         <v>5</v>
       </c>
       <c r="C164" t="s">
         <v>34</v>
       </c>
-      <c r="D164" s="1">
+      <c r="D164" s="3">
         <v>5045</v>
       </c>
       <c r="E164" t="s">
@@ -4318,13 +4326,13 @@
       <c r="A165" t="s">
         <v>190</v>
       </c>
-      <c r="B165" s="2">
+      <c r="B165" s="1">
         <v>5</v>
       </c>
       <c r="C165" t="s">
         <v>34</v>
       </c>
-      <c r="D165" s="1">
+      <c r="D165" s="3">
         <v>5147</v>
       </c>
       <c r="E165" t="s">
@@ -4335,13 +4343,13 @@
       <c r="A166" t="s">
         <v>190</v>
       </c>
-      <c r="B166" s="2">
+      <c r="B166" s="1">
         <v>5</v>
       </c>
       <c r="C166" t="s">
         <v>34</v>
       </c>
-      <c r="D166" s="1">
+      <c r="D166" s="3">
         <v>5172</v>
       </c>
       <c r="E166" t="s">
@@ -4352,13 +4360,13 @@
       <c r="A167" t="s">
         <v>190</v>
       </c>
-      <c r="B167" s="2">
+      <c r="B167" s="1">
         <v>5</v>
       </c>
       <c r="C167" t="s">
         <v>34</v>
       </c>
-      <c r="D167" s="1">
+      <c r="D167" s="3">
         <v>5234</v>
       </c>
       <c r="E167" t="s">
@@ -4369,13 +4377,13 @@
       <c r="A168" t="s">
         <v>190</v>
       </c>
-      <c r="B168" s="2">
+      <c r="B168" s="1">
         <v>5</v>
       </c>
       <c r="C168" t="s">
         <v>34</v>
       </c>
-      <c r="D168" s="1">
+      <c r="D168" s="3">
         <v>5480</v>
       </c>
       <c r="E168" t="s">
@@ -4386,13 +4394,13 @@
       <c r="A169" t="s">
         <v>190</v>
       </c>
-      <c r="B169" s="2">
+      <c r="B169" s="1">
         <v>5</v>
       </c>
       <c r="C169" t="s">
         <v>34</v>
       </c>
-      <c r="D169" s="1">
+      <c r="D169" s="3">
         <v>5490</v>
       </c>
       <c r="E169" t="s">
@@ -4403,13 +4411,13 @@
       <c r="A170" t="s">
         <v>190</v>
       </c>
-      <c r="B170" s="2">
+      <c r="B170" s="1">
         <v>5</v>
       </c>
       <c r="C170" t="s">
         <v>34</v>
       </c>
-      <c r="D170" s="1">
+      <c r="D170" s="3">
         <v>5665</v>
       </c>
       <c r="E170" t="s">
@@ -4420,13 +4428,13 @@
       <c r="A171" t="s">
         <v>190</v>
       </c>
-      <c r="B171" s="2">
+      <c r="B171" s="1">
         <v>5</v>
       </c>
       <c r="C171" t="s">
         <v>34</v>
       </c>
-      <c r="D171" s="1">
+      <c r="D171" s="3">
         <v>5837</v>
       </c>
       <c r="E171" t="s">

</xml_diff>